<commit_message>
E-COM TIP: episode titles 01-20 (new order, #01 = beautiful video) + planning sheet updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jo9AUb55boJfKH1RkCfDt9
</commit_message>
<xml_diff>
--- a/content/E-COM_TIP_planning.xlsx
+++ b/content/E-COM_TIP_planning.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="137" uniqueCount="111">
   <si>
     <t xml:space="preserve">سلسلة E-COM TIP — معلومة وحدة في كل فيديو  •  @kabli_ms</t>
   </si>
@@ -70,6 +70,27 @@
     <t xml:space="preserve">#01</t>
   </si>
   <si>
+    <t xml:space="preserve">فيديو شباب وما جابليش</t>
+  </si>
+  <si>
+    <t xml:space="preserve">فيديو شباب… بصح ما جابليش؟</t>
+  </si>
+  <si>
+    <t xml:space="preserve">الفيديو الشباب ماشي ديما يبيع: لازم يحبس الكليان في 3 ثواني ويفهم واش ينفعو</t>
+  </si>
+  <si>
+    <t xml:space="preserve">شوف واش اللي مبدّل عندك على الناس الأخرين وقولو من البداية</t>
+  </si>
+  <si>
+    <t xml:space="preserve">شحال من كليان 👥 · بدّل الفيديو 🔁 · لازم يحبسو ✋ · راحتلك البيعة 💸</t>
+  </si>
+  <si>
+    <t xml:space="preserve">مونتاج ✂️</t>
+  </si>
+  <si>
+    <t xml:space="preserve">#02</t>
+  </si>
+  <si>
     <t xml:space="preserve">Confirmation</t>
   </si>
   <si>
@@ -88,7 +109,7 @@
     <t xml:space="preserve">ما بديتش</t>
   </si>
   <si>
-    <t xml:space="preserve">#02</t>
+    <t xml:space="preserve">#03</t>
   </si>
   <si>
     <t xml:space="preserve">صور المنتوج</t>
@@ -106,7 +127,7 @@
     <t xml:space="preserve">صور حقيقية 📸 · confiance 🤝</t>
   </si>
   <si>
-    <t xml:space="preserve">#03</t>
+    <t xml:space="preserve">#04</t>
   </si>
   <si>
     <t xml:space="preserve">الربح الحقيقي</t>
@@ -124,7 +145,7 @@
     <t xml:space="preserve">الربح الحقيقي 💰 · pub · retours</t>
   </si>
   <si>
-    <t xml:space="preserve">#04</t>
+    <t xml:space="preserve">#05</t>
   </si>
   <si>
     <t xml:space="preserve">جاوب بالزربة</t>
@@ -142,7 +163,7 @@
     <t xml:space="preserve">جاوب بالزربة 💬</t>
   </si>
   <si>
-    <t xml:space="preserve">#05</t>
+    <t xml:space="preserve">#06</t>
   </si>
   <si>
     <t xml:space="preserve">هوك الإعلان</t>
@@ -160,7 +181,7 @@
     <t xml:space="preserve">3 ثواني ⏱️ · ابدا بالمشكل</t>
   </si>
   <si>
-    <t xml:space="preserve">#06</t>
+    <t xml:space="preserve">#07</t>
   </si>
   <si>
     <t xml:space="preserve">جرّب أكثر من إعلان</t>
@@ -178,7 +199,7 @@
     <t xml:space="preserve">test 🎬</t>
   </si>
   <si>
-    <t xml:space="preserve">#07</t>
+    <t xml:space="preserve">#08</t>
   </si>
   <si>
     <t xml:space="preserve">الإعلان الرابح</t>
@@ -196,7 +217,7 @@
     <t xml:space="preserve">ما تقيسوش ✋</t>
   </si>
   <si>
-    <t xml:space="preserve">#08</t>
+    <t xml:space="preserve">#09</t>
   </si>
   <si>
     <t xml:space="preserve">البيدجي بالشوية</t>
@@ -214,7 +235,7 @@
     <t xml:space="preserve">بالشوية 📈</t>
   </si>
   <si>
-    <t xml:space="preserve">#09</t>
+    <t xml:space="preserve">#10</t>
   </si>
   <si>
     <t xml:space="preserve">Pixel Meta</t>
@@ -232,7 +253,7 @@
     <t xml:space="preserve">Pixel Meta 🎯</t>
   </si>
   <si>
-    <t xml:space="preserve">#10</t>
+    <t xml:space="preserve">#11</t>
   </si>
   <si>
     <t xml:space="preserve">آراء الكليان</t>
@@ -250,7 +271,7 @@
     <t xml:space="preserve">آراء الكليان ⭐</t>
   </si>
   <si>
-    <t xml:space="preserve">#11</t>
+    <t xml:space="preserve">#12</t>
   </si>
   <si>
     <t xml:space="preserve">Offre / bundle</t>
@@ -262,7 +283,7 @@
     <t xml:space="preserve">(السكريبت من بعد)</t>
   </si>
   <si>
-    <t xml:space="preserve">#12</t>
+    <t xml:space="preserve">#13</t>
   </si>
   <si>
     <t xml:space="preserve">Livraison</t>
@@ -271,7 +292,7 @@
     <t xml:space="preserve">اختار société de livraison مليحة، الـ retour يكلفك</t>
   </si>
   <si>
-    <t xml:space="preserve">#13</t>
+    <t xml:space="preserve">#14</t>
   </si>
   <si>
     <t xml:space="preserve">Angle différent</t>
@@ -280,7 +301,7 @@
     <t xml:space="preserve">الموديل يتسرق، الطريقة تاعك ما تتسرقش</t>
   </si>
   <si>
-    <t xml:space="preserve">#14</t>
+    <t xml:space="preserve">#15</t>
   </si>
   <si>
     <t xml:space="preserve">ميساج التأكيد</t>
@@ -289,7 +310,7 @@
     <t xml:space="preserve">ميساج واتساب واحد ينقص الـ retours</t>
   </si>
   <si>
-    <t xml:space="preserve">#15</t>
+    <t xml:space="preserve">#16</t>
   </si>
   <si>
     <t xml:space="preserve">منتوج saturé</t>
@@ -298,7 +319,7 @@
     <t xml:space="preserve">المنتوج اللي راه عند الكل صعيب تربح فيه</t>
   </si>
   <si>
-    <t xml:space="preserve">#16</t>
+    <t xml:space="preserve">#17</t>
   </si>
   <si>
     <t xml:space="preserve">الاسم واللوغو</t>
@@ -307,7 +328,7 @@
     <t xml:space="preserve">ماركة بسيطة = ثقة أكثر</t>
   </si>
   <si>
-    <t xml:space="preserve">#17</t>
+    <t xml:space="preserve">#18</t>
   </si>
   <si>
     <t xml:space="preserve">وصف المنتوج</t>
@@ -316,7 +337,7 @@
     <t xml:space="preserve">اكتب الفايدة، ماشي غير المواصفات</t>
   </si>
   <si>
-    <t xml:space="preserve">#18</t>
+    <t xml:space="preserve">#19</t>
   </si>
   <si>
     <t xml:space="preserve">تتبّع الأرقام</t>
@@ -325,22 +346,13 @@
     <t xml:space="preserve">اكتب كل نهار: pub، commandes، retours</t>
   </si>
   <si>
-    <t xml:space="preserve">#19</t>
+    <t xml:space="preserve">#20</t>
   </si>
   <si>
     <t xml:space="preserve">Landing page</t>
   </si>
   <si>
     <t xml:space="preserve">ميساجات بزاف وكوموند قليلة؟ جرّب landing page</t>
-  </si>
-  <si>
-    <t xml:space="preserve">#20</t>
-  </si>
-  <si>
-    <t xml:space="preserve">آراء بالفيديو</t>
-  </si>
-  <si>
-    <t xml:space="preserve">فيديو كليان راضي يبني الثقة</t>
   </si>
 </sst>
 </file>
@@ -1030,27 +1042,27 @@
         <v>E-COM TIP #02</v>
       </c>
       <c r="J7" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B8" s="8" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C8" s="9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D8" s="9" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E8" s="9" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F8" s="9" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="G8" s="10" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H8),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1065,27 +1077,27 @@
         <v>E-COM TIP #03</v>
       </c>
       <c r="J8" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G9" s="16" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H9),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1100,27 +1112,27 @@
         <v>E-COM TIP #04</v>
       </c>
       <c r="J9" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B10" s="8" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E10" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F10" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G10" s="10" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H10),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1135,27 +1147,27 @@
         <v>E-COM TIP #05</v>
       </c>
       <c r="J10" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="B11" s="14" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G11" s="16" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H11),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1170,27 +1182,27 @@
         <v>E-COM TIP #06</v>
       </c>
       <c r="J11" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B12" s="8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C12" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E12" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="F12" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G12" s="10" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H12),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1205,27 +1217,27 @@
         <v>E-COM TIP #07</v>
       </c>
       <c r="J12" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B13" s="14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="G13" s="16" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H13),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1240,27 +1252,27 @@
         <v>E-COM TIP #08</v>
       </c>
       <c r="J13" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B14" s="8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G14" s="10" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H14),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1275,27 +1287,27 @@
         <v>E-COM TIP #09</v>
       </c>
       <c r="J14" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B15" s="14" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D15" s="15" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E15" s="15" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="F15" s="15" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G15" s="16" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H15),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
@@ -1310,24 +1322,28 @@
         <v>E-COM TIP #10</v>
       </c>
       <c r="J15" s="12" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="48" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="7" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B16" s="8" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C16" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
+        <v>80</v>
+      </c>
+      <c r="E16" s="9" t="s">
+        <v>81</v>
+      </c>
+      <c r="F16" s="9" t="s">
+        <v>82</v>
+      </c>
       <c r="G16" s="10" t="str">
         <f aca="false">CHOOSE(WEEKDAY(H16),"الأحد","الإثنين","الثلاثاء","الأربعاء","الخميس","الجمعة","السبت")</f>
         <v>الثلاثاء</v>
@@ -1341,21 +1357,21 @@
         <v>E-COM TIP #11</v>
       </c>
       <c r="J16" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="D17" s="15" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E17" s="15"/>
       <c r="F17" s="15"/>
@@ -1372,21 +1388,21 @@
         <v>E-COM TIP #12</v>
       </c>
       <c r="J17" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="7" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B18" s="8" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="C18" s="9" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E18" s="9"/>
       <c r="F18" s="9"/>
@@ -1403,21 +1419,21 @@
         <v>E-COM TIP #13</v>
       </c>
       <c r="J18" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
+        <v>90</v>
+      </c>
+      <c r="B19" s="14" t="s">
+        <v>91</v>
+      </c>
+      <c r="C19" s="15" t="s">
+        <v>92</v>
+      </c>
+      <c r="D19" s="15" t="s">
         <v>86</v>
-      </c>
-      <c r="B19" s="14" t="s">
-        <v>87</v>
-      </c>
-      <c r="C19" s="15" t="s">
-        <v>88</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>79</v>
       </c>
       <c r="E19" s="15"/>
       <c r="F19" s="15"/>
@@ -1434,21 +1450,21 @@
         <v>E-COM TIP #14</v>
       </c>
       <c r="J19" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="7" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="B20" s="8" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E20" s="9"/>
       <c r="F20" s="9"/>
@@ -1465,21 +1481,21 @@
         <v>E-COM TIP #15</v>
       </c>
       <c r="J20" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>93</v>
+        <v>97</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>94</v>
+        <v>98</v>
       </c>
       <c r="D21" s="15" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E21" s="15"/>
       <c r="F21" s="15"/>
@@ -1496,21 +1512,21 @@
         <v>E-COM TIP #16</v>
       </c>
       <c r="J21" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="7" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C22" s="9" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E22" s="9"/>
       <c r="F22" s="9"/>
@@ -1527,21 +1543,21 @@
         <v>E-COM TIP #17</v>
       </c>
       <c r="J22" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="D23" s="15" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E23" s="15"/>
       <c r="F23" s="15"/>
@@ -1558,21 +1574,21 @@
         <v>E-COM TIP #18</v>
       </c>
       <c r="J23" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="7" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="B24" s="8" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="C24" s="9" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E24" s="9"/>
       <c r="F24" s="9"/>
@@ -1589,21 +1605,21 @@
         <v>E-COM TIP #19</v>
       </c>
       <c r="J24" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="B25" s="14" t="s">
-        <v>105</v>
+        <v>109</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>106</v>
+        <v>110</v>
       </c>
       <c r="D25" s="15" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="E25" s="15"/>
       <c r="F25" s="15"/>
@@ -1620,7 +1636,7 @@
         <v>E-COM TIP #20</v>
       </c>
       <c r="J25" s="12" t="s">
-        <v>21</v>
+        <v>28</v>
       </c>
     </row>
   </sheetData>

</xml_diff>